<commit_message>
Refactoring to top-level DI
</commit_message>
<xml_diff>
--- a/WorkBot/refactor-experimental/data/orders/FingerLakes Farms/FingerLakes Farms_Collegetown_20251031.xlsx
+++ b/WorkBot/refactor-experimental/data/orders/FingerLakes Farms/FingerLakes Farms_Collegetown_20251031.xlsx
@@ -510,7 +510,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -520,7 +520,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>18.50</t>
+          <t>9.25</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>18.50</t>
+          <t>9.25</t>
         </is>
       </c>
     </row>

</xml_diff>